<commit_message>
update menu bulk modul head office 031125
</commit_message>
<xml_diff>
--- a/public/template/template_bulk_agi_ho.xlsx
+++ b/public/template/template_bulk_agi_ho.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data\Kerjaan\Bjb\Aplikasi AMT\Back Office\App\Local\bulk_kosongan\public\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA4444B8-A3B5-4186-BC11-A92AA61A3AF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C693199E-EBEF-4E93-9A8A-DC2548E00179}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -471,8 +471,8 @@
     <dataValidation type="textLength" operator="equal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Rekening Eksternal" error="Inputan tidak boleh kurang atau lebih dari 13 karakter." promptTitle="Input Validation" prompt="Inputan tidak boleh kurang atau lebih dari 13 karakter." sqref="B2:B1048576" xr:uid="{D63491A6-D9A0-4933-9436-9AC885D3830C}">
       <formula1>13</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Keterangan 1" error="Tidak diperbolehkan menggunakan spesial karakter * ? :  dan panjang teks tidak boleh melebihi 35 karakter." promptTitle="Input Validation" prompt="Tidak diperbolehkan menggunakan spesial karakter * ? :  dan panjang teks tidak boleh melebihi 35 karakter." sqref="I2:I1048576" xr:uid="{722273AA-008D-4AFB-9109-1516AC082185}">
-      <formula1>" =AND(ISERROR(FIND(""?"",I2)), ISERROR(FIND("":"",I2)), ISERROR(FIND(""*"",I2)), LEN(I2)&lt;=35)"</formula1>
+    <dataValidation type="custom" showInputMessage="1" showErrorMessage="1" errorTitle="Keterangan 1" error="Tidak diperbolehkan menggunakan spesial karakter * ? :  dan panjang teks tidak boleh melebihi 35 karakter." promptTitle="Input Validation" prompt="Tidak diperbolehkan menggunakan spesial karakter * ? :  dan panjang teks tidak boleh melebihi 35 karakter." sqref="I2:I1048576" xr:uid="{722273AA-008D-4AFB-9109-1516AC082185}">
+      <formula1>AND(ISERROR(FIND("?",I2)), ISERROR(FIND(":",I2)), ISERROR(FIND("*",I2)), LEN(I2)&lt;=35)</formula1>
     </dataValidation>
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Keterangan 2" error="Tidak diperbolehkan menggunakan spesial karakter * ? :  dan panjang teks tidak boleh melebihi 35 karakter." promptTitle="Input Validation" prompt="Tidak diperbolehkan menggunakan spesial karakter * ? :  dan panjang teks tidak boleh melebihi 35 karakter." sqref="J2:J1048576" xr:uid="{2602352D-8A01-4165-9A7F-0D398AC81B79}">
       <formula1>AND(ISERROR(FIND("?",J2)), ISERROR(FIND(":",J2)), ISERROR(FIND("*",J2)), LEN(J2)&lt;=35)</formula1>

</xml_diff>